<commit_message>
reproduce the original text
</commit_message>
<xml_diff>
--- a/strategy_Result.xlsx
+++ b/strategy_Result.xlsx
@@ -346,7 +346,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1">
         <v>1</v>
@@ -358,7 +358,7 @@
         <v>0</v>
       </c>
       <c r="E1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F1">
         <v>1</v>
@@ -367,7 +367,7 @@
         <v>1</v>
       </c>
       <c r="H1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1">
         <v>0</v>
@@ -382,7 +382,7 @@
         <v>1</v>
       </c>
       <c r="M1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N1">
         <v>1</v>
@@ -391,7 +391,7 @@
         <v>1</v>
       </c>
       <c r="P1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q1">
         <v>1</v>
@@ -411,10 +411,10 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -432,19 +432,19 @@
         <v>1</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -453,13 +453,13 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2">
         <v>1</v>
@@ -470,13 +470,13 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -488,22 +488,22 @@
         <v>1</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3">
         <v>1</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3">
         <v>1</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M3">
         <v>1</v>
@@ -521,24 +521,24 @@
         <v>1</v>
       </c>
       <c r="R3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S3">
         <v>1</v>
       </c>
       <c r="T3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:20">
       <c r="A4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -547,7 +547,7 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -559,10 +559,10 @@
         <v>1</v>
       </c>
       <c r="J4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L4">
         <v>1</v>
@@ -571,7 +571,7 @@
         <v>1</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O4">
         <v>1</v>
@@ -589,7 +589,7 @@
         <v>1</v>
       </c>
       <c r="T4">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -600,7 +600,7 @@
         <v>1</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -609,49 +609,49 @@
         <v>1</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5">
         <v>1</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L5">
         <v>0</v>
       </c>
       <c r="M5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O5">
         <v>1</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R5">
         <v>1</v>
       </c>
       <c r="S5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -662,7 +662,7 @@
         <v>1</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -674,7 +674,7 @@
         <v>1</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -689,7 +689,7 @@
         <v>1</v>
       </c>
       <c r="L6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M6">
         <v>1</v>
@@ -701,16 +701,16 @@
         <v>0</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R6">
         <v>1</v>
       </c>
       <c r="S6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T6">
         <v>1</v>
@@ -721,10 +721,10 @@
         <v>1</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -742,13 +742,13 @@
         <v>1</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L7">
         <v>1</v>
@@ -766,10 +766,10 @@
         <v>1</v>
       </c>
       <c r="Q7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S7">
         <v>1</v>
@@ -792,7 +792,7 @@
         <v>1</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -801,10 +801,10 @@
         <v>1</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8">
         <v>1</v>
@@ -822,16 +822,16 @@
         <v>1</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q8">
         <v>1</v>
       </c>
       <c r="R8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S8">
         <v>1</v>
@@ -857,19 +857,19 @@
         <v>1</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9">
         <v>1</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9">
         <v>1</v>
       </c>
       <c r="J9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9">
         <v>1</v>
@@ -887,16 +887,16 @@
         <v>1</v>
       </c>
       <c r="P9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R9">
         <v>1</v>
       </c>
       <c r="S9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T9">
         <v>1</v>
@@ -904,7 +904,7 @@
     </row>
     <row r="10" spans="1:20">
       <c r="A10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -916,7 +916,7 @@
         <v>1</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10">
         <v>1</v>
@@ -940,19 +940,19 @@
         <v>1</v>
       </c>
       <c r="M10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P10">
         <v>0</v>
       </c>
       <c r="Q10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R10">
         <v>1</v>
@@ -966,16 +966,16 @@
     </row>
     <row r="11" spans="1:20">
       <c r="A11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -987,7 +987,7 @@
         <v>1</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I11">
         <v>1</v>
@@ -1040,7 +1040,7 @@
         <v>1</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12">
         <v>1</v>
@@ -1052,7 +1052,7 @@
         <v>1</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J12">
         <v>1</v>
@@ -1061,10 +1061,10 @@
         <v>1</v>
       </c>
       <c r="L12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N12">
         <v>1</v>
@@ -1093,7 +1093,7 @@
         <v>1</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -1111,13 +1111,13 @@
         <v>1</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13">
         <v>1</v>
@@ -1126,7 +1126,7 @@
         <v>0</v>
       </c>
       <c r="M13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N13">
         <v>1</v>
@@ -1135,16 +1135,16 @@
         <v>1</v>
       </c>
       <c r="P13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R13">
         <v>1</v>
       </c>
       <c r="S13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T13">
         <v>0</v>
@@ -1155,16 +1155,16 @@
         <v>1</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14">
         <v>1</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -1173,10 +1173,10 @@
         <v>1</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14">
         <v>1</v>
@@ -1214,16 +1214,16 @@
     </row>
     <row r="15" spans="1:20">
       <c r="A15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -1232,7 +1232,7 @@
         <v>1</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15">
         <v>1</v>
@@ -1241,22 +1241,22 @@
         <v>1</v>
       </c>
       <c r="J15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15">
         <v>1</v>
       </c>
       <c r="L15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M15">
         <v>1</v>
       </c>
       <c r="N15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P15">
         <v>1</v>
@@ -1279,19 +1279,19 @@
         <v>1</v>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -1303,16 +1303,16 @@
         <v>1</v>
       </c>
       <c r="J16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N16">
         <v>1</v>
@@ -1327,7 +1327,7 @@
         <v>1</v>
       </c>
       <c r="R16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16">
         <v>1</v>
@@ -1338,10 +1338,10 @@
     </row>
     <row r="17" spans="1:20">
       <c r="A17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -1350,7 +1350,7 @@
         <v>1</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17">
         <v>1</v>
@@ -1371,7 +1371,7 @@
         <v>1</v>
       </c>
       <c r="L17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M17">
         <v>1</v>
@@ -1386,10 +1386,10 @@
         <v>1</v>
       </c>
       <c r="Q17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S17">
         <v>1</v>
@@ -1406,7 +1406,7 @@
         <v>0</v>
       </c>
       <c r="C18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -1415,31 +1415,31 @@
         <v>1</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18">
         <v>0</v>
       </c>
       <c r="H18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I18">
         <v>1</v>
       </c>
       <c r="J18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18">
         <v>1</v>
       </c>
       <c r="L18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M18">
         <v>0</v>
       </c>
       <c r="N18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O18">
         <v>1</v>
@@ -1462,22 +1462,22 @@
     </row>
     <row r="19" spans="1:20">
       <c r="A19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19">
         <v>0</v>
       </c>
       <c r="F19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -1486,22 +1486,22 @@
         <v>1</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O19">
         <v>1</v>
@@ -1527,7 +1527,7 @@
         <v>1</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -1536,7 +1536,7 @@
         <v>1</v>
       </c>
       <c r="E20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20">
         <v>1</v>
@@ -1554,7 +1554,7 @@
         <v>1</v>
       </c>
       <c r="K20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L20">
         <v>0</v>
@@ -1596,10 +1596,10 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="C1">
         <v>0</v>
@@ -1608,16 +1608,16 @@
         <v>0</v>
       </c>
       <c r="E1">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F1">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G1">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="H1">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I1">
         <v>0</v>
@@ -1626,13 +1626,13 @@
         <v>1</v>
       </c>
       <c r="K1">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="L1">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="M1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N1">
         <v>-1</v>
@@ -1641,13 +1641,13 @@
         <v>-1</v>
       </c>
       <c r="P1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q1">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="R1">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S1">
         <v>1</v>
@@ -1661,40 +1661,40 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G2">
         <v>-1</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1</v>
       </c>
       <c r="L2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -1703,16 +1703,16 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="T2">
         <v>1</v>
@@ -1720,46 +1720,46 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3">
         <v>1</v>
       </c>
       <c r="L3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="N3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="O3">
         <v>1</v>
@@ -1768,60 +1768,60 @@
         <v>1</v>
       </c>
       <c r="Q3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="R3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="T3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:20">
       <c r="A4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="H4">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I4">
         <v>1</v>
       </c>
       <c r="J4">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K4">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="L4">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="M4">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O4">
         <v>1</v>
@@ -1830,16 +1830,16 @@
         <v>0</v>
       </c>
       <c r="Q4">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="R4">
         <v>0</v>
       </c>
       <c r="S4">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="T4">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -1847,90 +1847,90 @@
         <v>-1</v>
       </c>
       <c r="B5">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5">
         <v>-1</v>
       </c>
       <c r="E5">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I5">
         <v>-1</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="L5">
         <v>0</v>
       </c>
       <c r="M5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O5">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R5">
         <v>1</v>
       </c>
       <c r="S5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:20">
       <c r="A6">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E6">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="J6">
         <v>-1</v>
@@ -1939,28 +1939,28 @@
         <v>-1</v>
       </c>
       <c r="L6">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="M6">
         <v>1</v>
       </c>
       <c r="N6">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R6">
         <v>1</v>
       </c>
       <c r="S6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T6">
         <v>-1</v>
@@ -1971,10 +1971,10 @@
         <v>-1</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7">
         <v>-1</v>
@@ -1983,22 +1983,22 @@
         <v>0</v>
       </c>
       <c r="F7">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G7">
         <v>1</v>
       </c>
       <c r="H7">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L7">
         <v>1</v>
@@ -2013,16 +2013,16 @@
         <v>1</v>
       </c>
       <c r="P7">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Q7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S7">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="T7">
         <v>-1</v>
@@ -2030,19 +2030,19 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="C8">
         <v>-1</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -2051,37 +2051,37 @@
         <v>1</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="K8">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="L8">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="M8">
         <v>1</v>
       </c>
       <c r="N8">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q8">
         <v>1</v>
       </c>
       <c r="R8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S8">
         <v>1</v>
@@ -2107,54 +2107,54 @@
         <v>-1</v>
       </c>
       <c r="F9">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G9">
         <v>1</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="J9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="N9">
         <v>1</v>
       </c>
       <c r="O9">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="P9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q9">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R9">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T9">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="10" spans="1:20">
       <c r="A10">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="B10">
         <v>-1</v>
@@ -2166,10 +2166,10 @@
         <v>-1</v>
       </c>
       <c r="E10">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F10">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G10">
         <v>1</v>
@@ -2181,84 +2181,84 @@
         <v>1</v>
       </c>
       <c r="J10">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="K10">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="L10">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="M10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N10">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="O10">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="P10">
         <v>0</v>
       </c>
       <c r="Q10">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="R10">
         <v>1</v>
       </c>
       <c r="S10">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="T10">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="11" spans="1:20">
       <c r="A11">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="B11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E11">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="F11">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="H11">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I11">
         <v>1</v>
       </c>
       <c r="J11">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="K11">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="N11">
         <v>-1</v>
       </c>
       <c r="O11">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="P11">
         <v>-1</v>
@@ -2270,7 +2270,7 @@
         <v>-1</v>
       </c>
       <c r="S11">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="T11">
         <v>0</v>
@@ -2278,46 +2278,46 @@
     </row>
     <row r="12" spans="1:20">
       <c r="A12">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12">
         <v>-1</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I12">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J12">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="K12">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="L12">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="M12">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="N12">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="O12">
         <v>-1</v>
@@ -2329,13 +2329,13 @@
         <v>-1</v>
       </c>
       <c r="R12">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S12">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="T12">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -2343,13 +2343,13 @@
         <v>-1</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E13">
         <v>-1</v>
@@ -2358,43 +2358,43 @@
         <v>-1</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K13">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="L13">
         <v>0</v>
       </c>
       <c r="M13">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="N13">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="O13">
         <v>-1</v>
       </c>
       <c r="P13">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="Q13">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="R13">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S13">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T13">
         <v>0</v>
@@ -2405,16 +2405,16 @@
         <v>-1</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -2423,13 +2423,13 @@
         <v>-1</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="K14">
         <v>1</v>
@@ -2441,10 +2441,10 @@
         <v>-1</v>
       </c>
       <c r="N14">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="O14">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="P14">
         <v>-1</v>
@@ -2453,66 +2453,66 @@
         <v>-1</v>
       </c>
       <c r="R14">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S14">
         <v>-1</v>
       </c>
       <c r="T14">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15">
         <v>-1</v>
       </c>
       <c r="F15">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I15">
         <v>-1</v>
       </c>
       <c r="J15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15">
         <v>1</v>
       </c>
       <c r="L15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M15">
         <v>-1</v>
       </c>
       <c r="N15">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="O15">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="P15">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Q15">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="R15">
         <v>-1</v>
@@ -2526,176 +2526,176 @@
     </row>
     <row r="16" spans="1:20">
       <c r="A16">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="B16">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G16">
         <v>-1</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="J16">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="K16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N16">
         <v>1</v>
       </c>
       <c r="O16">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="P16">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Q16">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="R16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16">
         <v>-1</v>
       </c>
       <c r="T16">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="17" spans="1:20">
       <c r="A17">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C17">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="D17">
         <v>1</v>
       </c>
       <c r="E17">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F17">
         <v>-1</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="H17">
         <v>0</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="J17">
         <v>-1</v>
       </c>
       <c r="K17">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="L17">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="M17">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="N17">
         <v>1</v>
       </c>
       <c r="O17">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="P17">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Q17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S17">
         <v>-1</v>
       </c>
       <c r="T17">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="18" spans="1:20">
       <c r="A18">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="B18">
         <v>0</v>
       </c>
       <c r="C18">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
       <c r="E18">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18">
         <v>0</v>
       </c>
       <c r="H18">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I18">
         <v>-1</v>
       </c>
       <c r="J18">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="K18">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="L18">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="M18">
         <v>0</v>
       </c>
       <c r="N18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O18">
         <v>1</v>
       </c>
       <c r="P18">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Q18">
         <v>1</v>
@@ -2704,7 +2704,7 @@
         <v>0</v>
       </c>
       <c r="S18">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="T18">
         <v>-1</v>
@@ -2712,81 +2712,81 @@
     </row>
     <row r="19" spans="1:20">
       <c r="A19">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="B19">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="C19">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="D19">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E19">
         <v>0</v>
       </c>
       <c r="F19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="H19">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J19">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="K19">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="L19">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="M19">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="N19">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="O19">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="P19">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Q19">
         <v>0</v>
       </c>
       <c r="R19">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S19">
         <v>1</v>
       </c>
       <c r="T19">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:20">
       <c r="A20">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="B20">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E20">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F20">
         <v>-1</v>
@@ -2804,7 +2804,7 @@
         <v>1</v>
       </c>
       <c r="K20">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="L20">
         <v>0</v>
@@ -2816,7 +2816,7 @@
         <v>-1</v>
       </c>
       <c r="O20">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="P20">
         <v>-1</v>
@@ -2831,7 +2831,7 @@
         <v>1</v>
       </c>
       <c r="T20">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>